<commit_message>
chore: fix testcase ID format
</commit_message>
<xml_diff>
--- a/test-cases/demoblaze-test-cases.xlsx
+++ b/test-cases/demoblaze-test-cases.xlsx
@@ -442,7 +442,7 @@
   <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -515,7 +515,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-001</t>
+          <t>TC-001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-002</t>
+          <t>TC-002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-003</t>
+          <t>TC-003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-004</t>
+          <t>TC-004</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -727,7 +727,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-005</t>
+          <t>TC-005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -776,7 +776,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-006</t>
+          <t>TC-006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-007</t>
+          <t>TC-007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TC-LOGIN-008</t>
+          <t>TC-008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TC-CART-001</t>
+          <t>TC-009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TC-CART-002</t>
+          <t>TC-010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1025,7 +1025,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TC-CART-003</t>
+          <t>TC-011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TC-CART-004</t>
+          <t>TC-012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1123,7 +1123,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TC-CART-005</t>
+          <t>TC-013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-ORDER-001</t>
+          <t>TC-014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1225,7 +1225,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TC-ORDER-002</t>
+          <t>TC-015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1278,7 +1278,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TC-ORDER-003</t>
+          <t>TC-016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1331,7 +1331,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TC-ORDER-004</t>
+          <t>TC-017</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1384,7 +1384,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>TC-ORDER-005</t>
+          <t>TC-018</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1441,7 +1441,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>TC-ORDER-006</t>
+          <t>TC-019</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">

</xml_diff>

<commit_message>
chore: minor fix testcase
</commit_message>
<xml_diff>
--- a/test-cases/demoblaze-test-cases.xlsx
+++ b/test-cases/demoblaze-test-cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luha/my_project/Playwright_Demo/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7056166A-6E19-EA4B-9B90-2E4D7E996947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFAA953-32C2-F44E-B5B6-11A7FE6AABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,9 +73,6 @@
 4. Click "Log in".</t>
   </si>
   <si>
-    <t>No alert. Navbar shows "Welcome &lt;username&gt;"; the "Log in" link is hidden.</t>
-  </si>
-  <si>
     <t>Y</t>
   </si>
   <si>
@@ -278,6 +275,9 @@
   </si>
   <si>
     <t>Correct behavior: the order should be blocked, or at minimum the amount should not be a real charge. Actual (defect): order succeeds, confirmation shows "Amount: 0 USD".</t>
+  </si>
+  <si>
+    <t>No alert. Navbar shows "Welcome &lt;username&gt;"</t>
   </si>
 </sst>
 </file>
@@ -708,82 +708,82 @@
         <v>15</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>13</v>
@@ -792,50 +792,50 @@
         <v>14</v>
       </c>
       <c r="G5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -844,88 +844,88 @@
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="3" t="s">
-        <v>42</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="G9" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>53</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>12</v>
@@ -934,132 +934,132 @@
         <v>13</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="I10" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G12" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="H12" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="H13" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="C14" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="I14" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
chore: update testcases to latest
</commit_message>
<xml_diff>
--- a/test-cases/demoblaze-test-cases.xlsx
+++ b/test-cases/demoblaze-test-cases.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luha/my_project/Playwright_Demo/test-cases/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFAA953-32C2-F44E-B5B6-11A7FE6AABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="34560" windowHeight="19320"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Test Cases" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="100">
   <si>
     <t>ID</t>
   </si>
@@ -67,12 +61,15 @@
     <t>A registered account exists</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Log in".
 3. Enter the account's username and password.
 4. Click "Log in".</t>
   </si>
   <si>
+    <t>No alert. Navbar shows "Welcome &lt;username&gt;"</t>
+  </si>
+  <si>
     <t>Y</t>
   </si>
   <si>
@@ -88,7 +85,7 @@
     <t>None</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Log in".
 3. Leave username and password empty.
 4. Click "Log in".</t>
@@ -103,7 +100,7 @@
     <t>Verify unknown username rejects with "User does not exist."</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Log in".
 3. Enter a username that has never been registered.
 4. Click "Log in".</t>
@@ -118,7 +115,7 @@
     <t>Verify wrong password rejects with "Wrong password."</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Log in".
 3. Enter the account's username with an incorrect password.
 4. Click "Log in".</t>
@@ -139,7 +136,7 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Sign up".
 3. Enter a username that is already registered.
 4. Click "Sign up".</t>
@@ -157,7 +154,7 @@
     <t>Verify user can sign up with a new unique username</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Sign up".
 3. Enter a brand-new unique username and a password.
 4. Click "Sign up".</t>
@@ -175,7 +172,7 @@
     <t>Low</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Sign up".
 3. Enter a very long username (200+ characters).
 4. Click "Sign up".</t>
@@ -190,7 +187,7 @@
     <t>Verify sign up with an empty password shows validation alert</t>
   </si>
   <si>
-    <t>1. Go to home page.
+    <t xml:space="preserve">1. Go to home page.
 2. Click "Sign up".
 3. Enter empty password
 4. Click "Sign up".</t>
@@ -208,7 +205,7 @@
     <t>Logged in, 1 item in cart</t>
   </si>
   <si>
-    <t>1. Go to Cart page.
+    <t xml:space="preserve">1. Go to Cart page.
 2. Click "Place Order".
 3. Fill in Name and Card only.
 4. Click "Purchase".</t>
@@ -226,7 +223,7 @@
     <t>Logged in</t>
   </si>
   <si>
-    <t>1. Go to Cart page.
+    <t xml:space="preserve">1. Go to Cart page.
 2. Click "Place Order".
 3. Leave Name and Card empty.
 4. Click "Purchase".</t>
@@ -241,7 +238,7 @@
     <t>Verify missing Name only shows the same validation alert</t>
   </si>
   <si>
-    <t>1. Go to Cart page.
+    <t xml:space="preserve">1. Go to Cart page.
 2. Click "Place Order".
 3. Fill Card only, leave Name empty.
 4. Click "Purchase".</t>
@@ -253,7 +250,7 @@
     <t>Verify missing Card only shows the same validation alert</t>
   </si>
   <si>
-    <t>1. Go to Cart page.
+    <t xml:space="preserve">1. Go to Cart page.
 2. Click "Place Order".
 3. Fill Name only, leave Card empty.
 4. Click "Purchase".</t>
@@ -268,7 +265,7 @@
     <t>Logged in, cart empty</t>
   </si>
   <si>
-    <t>1. Go to Cart page with an empty cart.
+    <t xml:space="preserve">1. Go to Cart page with an empty cart.
 2. Click "Place Order".
 3. Fill Name and Card.
 4. Click "Purchase".</t>
@@ -277,36 +274,119 @@
     <t>Correct behavior: the order should be blocked, or at minimum the amount should not be a real charge. Actual (defect): order succeeds, confirmation shows "Amount: 0 USD".</t>
   </si>
   <si>
-    <t>No alert. Navbar shows "Welcome &lt;username&gt;"</t>
+    <t>TC-014</t>
+  </si>
+  <si>
+    <t>Verify logged-in user can add a product to cart</t>
+  </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to home page.
+2. Open a product page.
+3. Click "Add to cart".
+4. Go to Cart page.</t>
+  </si>
+  <si>
+    <t>Alert: "Product added." Cart shows 1 row with the product name and price. Total equals that price.</t>
+  </si>
+  <si>
+    <t>TC-015</t>
+  </si>
+  <si>
+    <t>Verify adding two different products lists both with the summed total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Add product A to cart.
+2. Add product B to cart.
+3. Go to Cart page.</t>
+  </si>
+  <si>
+    <t>Cart shows 2 rows (A and B). Total equals the sum of both prices.</t>
+  </si>
+  <si>
+    <t>TC-016</t>
+  </si>
+  <si>
+    <t>Verify adding the same product twice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Add product A to cart.
+2. Add product A to cart again.
+3. Go to Cart page.</t>
+  </si>
+  <si>
+    <t>Cart shows 2 separate rows for product A. Total equals double the price.</t>
+  </si>
+  <si>
+    <t>TC-017</t>
+  </si>
+  <si>
+    <t>Verify user can delete the only item in the cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to Cart page.
+2. Click "Delete" on the item.</t>
+  </si>
+  <si>
+    <t>Page reloads. Cart is empty and the total is cleared.</t>
+  </si>
+  <si>
+    <t>TC-018</t>
+  </si>
+  <si>
+    <t>Verify deleting one of two items keeps the other and updates the total</t>
+  </si>
+  <si>
+    <t>Logged in, 2 different items in cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to Cart page.
+2. Click "Delete" on one item.</t>
+  </si>
+  <si>
+    <t>Page reloads. 1 row remains. Total equals the remaining item's price.</t>
+  </si>
+  <si>
+    <t>TC-019</t>
+  </si>
+  <si>
+    <t>Verify cart items persist after a page refresh</t>
+  </si>
+  <si>
+    <t>Logged in, 1 or more items in cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to Cart page.
+2. Refresh the page.</t>
+  </si>
+  <si>
+    <t>Same rows and same total are shown after the refresh.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <sz val="11"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -329,7 +409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -338,15 +418,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -642,9 +719,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
@@ -656,7 +733,7 @@
     <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -685,11 +762,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -708,82 +785,82 @@
         <v>15</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="4" t="s">
         <v>18</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="4" t="s">
         <v>24</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="4" t="s">
         <v>28</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>13</v>
@@ -792,50 +869,50 @@
         <v>14</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="4" t="s">
         <v>32</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="4" t="s">
         <v>39</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -844,88 +921,88 @@
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="4" t="s">
         <v>43</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="4" t="s">
         <v>48</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="4" t="s">
         <v>51</v>
       </c>
+      <c r="B10" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="C10" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>12</v>
@@ -934,152 +1011,310 @@
         <v>13</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>52</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="G12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" s="4" t="s">
         <v>65</v>
       </c>
+      <c r="B13" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="C13" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="4" t="s">
         <v>68</v>
       </c>
+      <c r="B14" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="C14" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G14" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="2"/>
-    </row>
-    <row r="16" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="17" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="18" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" ht="60" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="20" ht="45" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="G16" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>